<commit_message>
Add supported device models list
</commit_message>
<xml_diff>
--- a/doc/Bluetti-Open-Modbus-TCP-register-list-20260522.xlsx
+++ b/doc/Bluetti-Open-Modbus-TCP-register-list-20260522.xlsx
@@ -4,12 +4,13 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="27945" windowHeight="11805"/>
+    <workbookView windowWidth="27945" windowHeight="12255"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="19" r:id="rId1"/>
     <sheet name="Update Record" sheetId="14" r:id="rId2"/>
-    <sheet name="Meter" sheetId="16" r:id="rId3"/>
+    <sheet name="Device list" sheetId="20" r:id="rId3"/>
+    <sheet name="Meter" sheetId="16" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -29,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="120">
   <si>
     <t>Overview</t>
   </si>
@@ -76,8 +77,7 @@
     <t>None</t>
   </si>
   <si>
-    <t>1~247
-100:汇总数据</t>
+    <t>1~255 250:Summarize data</t>
   </si>
   <si>
     <t>Protocol Specification</t>
@@ -205,6 +205,33 @@
   </si>
   <si>
     <t>2026.05.22</t>
+  </si>
+  <si>
+    <t>Device Model</t>
+  </si>
+  <si>
+    <t>Modbus TCP Support</t>
+  </si>
+  <si>
+    <t>Webserver Configuration Support</t>
+  </si>
+  <si>
+    <t>Register Address Range</t>
+  </si>
+  <si>
+    <t>Firmware Version</t>
+  </si>
+  <si>
+    <t>SMeter</t>
+  </si>
+  <si>
+    <t>YES</t>
+  </si>
+  <si>
+    <t>read:55101~55300</t>
+  </si>
+  <si>
+    <t>EBOX</t>
   </si>
   <si>
     <t>Cassandra register list</t>
@@ -565,7 +592,7 @@
       <charset val="134"/>
     </font>
   </fonts>
-  <fills count="38">
+  <fills count="39">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -599,6 +626,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -929,10 +962,10 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right/>
+      <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
       <top style="thin">
         <color auto="1"/>
       </top>
@@ -942,10 +975,10 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
       <top style="thin">
         <color auto="1"/>
       </top>
@@ -1122,7 +1155,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="18" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="18" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1146,16 +1179,16 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="8" borderId="21" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="9" borderId="22" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="9" borderId="21" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="10" borderId="23" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="9" borderId="21" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="10" borderId="22" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="10" borderId="21" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="11" borderId="23" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="24" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
@@ -1164,92 +1197,92 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="25" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1305,6 +1338,10 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1345,7 +1382,22 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1353,25 +1405,7 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1713,633 +1747,633 @@
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <sheetData>
     <row r="1" spans="1:21">
-      <c r="A1" s="22"/>
-      <c r="B1" s="23"/>
-      <c r="C1" s="23"/>
-      <c r="D1" s="23"/>
-      <c r="E1" s="23"/>
-      <c r="F1" s="23"/>
-      <c r="G1" s="23"/>
-      <c r="H1" s="23"/>
-      <c r="I1" s="23"/>
-      <c r="J1" s="23"/>
-      <c r="K1" s="23"/>
-      <c r="L1" s="23"/>
-      <c r="M1" s="23"/>
-      <c r="N1" s="23"/>
-      <c r="O1" s="23"/>
-      <c r="P1" s="23"/>
-      <c r="Q1" s="23"/>
-      <c r="R1" s="23"/>
-      <c r="S1" s="23"/>
-      <c r="T1" s="23"/>
-      <c r="U1" s="24"/>
+      <c r="A1" s="24"/>
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="25"/>
+      <c r="G1" s="25"/>
+      <c r="H1" s="25"/>
+      <c r="I1" s="25"/>
+      <c r="J1" s="25"/>
+      <c r="K1" s="25"/>
+      <c r="L1" s="25"/>
+      <c r="M1" s="25"/>
+      <c r="N1" s="25"/>
+      <c r="O1" s="25"/>
+      <c r="P1" s="25"/>
+      <c r="Q1" s="25"/>
+      <c r="R1" s="25"/>
+      <c r="S1" s="25"/>
+      <c r="T1" s="25"/>
+      <c r="U1" s="26"/>
     </row>
     <row r="2" ht="15" customHeight="1" spans="1:21">
-      <c r="A2" s="25" t="s">
+      <c r="A2" s="27" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="25"/>
-      <c r="C2" s="25"/>
-      <c r="D2" s="25"/>
-      <c r="E2" s="25"/>
-      <c r="F2" s="25"/>
-      <c r="G2" s="25"/>
-      <c r="H2" s="25"/>
-      <c r="I2" s="25"/>
-      <c r="J2" s="25"/>
-      <c r="K2" s="26"/>
-      <c r="L2" s="26"/>
-      <c r="M2" s="26"/>
-      <c r="N2" s="26"/>
-      <c r="O2" s="26"/>
-      <c r="P2" s="26"/>
-      <c r="Q2" s="27"/>
-      <c r="R2" s="27"/>
-      <c r="S2" s="27"/>
-      <c r="T2" s="27"/>
-      <c r="U2" s="28"/>
+      <c r="B2" s="27"/>
+      <c r="C2" s="27"/>
+      <c r="D2" s="27"/>
+      <c r="E2" s="27"/>
+      <c r="F2" s="27"/>
+      <c r="G2" s="27"/>
+      <c r="H2" s="27"/>
+      <c r="I2" s="27"/>
+      <c r="J2" s="27"/>
+      <c r="K2" s="28"/>
+      <c r="L2" s="28"/>
+      <c r="M2" s="28"/>
+      <c r="N2" s="28"/>
+      <c r="O2" s="28"/>
+      <c r="P2" s="28"/>
+      <c r="Q2" s="29"/>
+      <c r="R2" s="29"/>
+      <c r="S2" s="29"/>
+      <c r="T2" s="29"/>
+      <c r="U2" s="30"/>
     </row>
     <row r="3" ht="15" customHeight="1" spans="1:21">
-      <c r="A3" s="29" t="s">
+      <c r="A3" s="31" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="29"/>
-      <c r="C3" s="29"/>
-      <c r="D3" s="29"/>
-      <c r="E3" s="29"/>
-      <c r="F3" s="29"/>
-      <c r="G3" s="29"/>
-      <c r="H3" s="29"/>
-      <c r="I3" s="29"/>
-      <c r="J3" s="29"/>
-      <c r="K3" s="26"/>
-      <c r="L3" s="26"/>
-      <c r="M3" s="26"/>
-      <c r="N3" s="26"/>
-      <c r="O3" s="26"/>
-      <c r="P3" s="26"/>
-      <c r="Q3" s="27"/>
-      <c r="R3" s="27"/>
-      <c r="S3" s="27"/>
-      <c r="T3" s="27"/>
-      <c r="U3" s="28"/>
+      <c r="B3" s="31"/>
+      <c r="C3" s="31"/>
+      <c r="D3" s="31"/>
+      <c r="E3" s="31"/>
+      <c r="F3" s="31"/>
+      <c r="G3" s="31"/>
+      <c r="H3" s="31"/>
+      <c r="I3" s="31"/>
+      <c r="J3" s="31"/>
+      <c r="K3" s="28"/>
+      <c r="L3" s="28"/>
+      <c r="M3" s="28"/>
+      <c r="N3" s="28"/>
+      <c r="O3" s="28"/>
+      <c r="P3" s="28"/>
+      <c r="Q3" s="29"/>
+      <c r="R3" s="29"/>
+      <c r="S3" s="29"/>
+      <c r="T3" s="29"/>
+      <c r="U3" s="30"/>
     </row>
     <row r="4" ht="15" customHeight="1" spans="1:21">
-      <c r="A4" s="29"/>
-      <c r="B4" s="29"/>
-      <c r="C4" s="29"/>
-      <c r="D4" s="29"/>
-      <c r="E4" s="29"/>
-      <c r="F4" s="29"/>
-      <c r="G4" s="29"/>
-      <c r="H4" s="29"/>
-      <c r="I4" s="29"/>
-      <c r="J4" s="29"/>
-      <c r="K4" s="26"/>
-      <c r="L4" s="26"/>
-      <c r="M4" s="26"/>
-      <c r="N4" s="26"/>
-      <c r="O4" s="26"/>
-      <c r="P4" s="26"/>
-      <c r="Q4" s="27"/>
-      <c r="R4" s="27"/>
-      <c r="S4" s="27"/>
-      <c r="T4" s="27"/>
-      <c r="U4" s="28"/>
+      <c r="A4" s="31"/>
+      <c r="B4" s="31"/>
+      <c r="C4" s="31"/>
+      <c r="D4" s="31"/>
+      <c r="E4" s="31"/>
+      <c r="F4" s="31"/>
+      <c r="G4" s="31"/>
+      <c r="H4" s="31"/>
+      <c r="I4" s="31"/>
+      <c r="J4" s="31"/>
+      <c r="K4" s="28"/>
+      <c r="L4" s="28"/>
+      <c r="M4" s="28"/>
+      <c r="N4" s="28"/>
+      <c r="O4" s="28"/>
+      <c r="P4" s="28"/>
+      <c r="Q4" s="29"/>
+      <c r="R4" s="29"/>
+      <c r="S4" s="29"/>
+      <c r="T4" s="29"/>
+      <c r="U4" s="30"/>
     </row>
     <row r="5" ht="15" customHeight="1" spans="1:21">
-      <c r="A5" s="29"/>
-      <c r="B5" s="29"/>
-      <c r="C5" s="29"/>
-      <c r="D5" s="29"/>
-      <c r="E5" s="29"/>
-      <c r="F5" s="29"/>
-      <c r="G5" s="29"/>
-      <c r="H5" s="29"/>
-      <c r="I5" s="29"/>
-      <c r="J5" s="29"/>
-      <c r="K5" s="26"/>
-      <c r="L5" s="26"/>
-      <c r="M5" s="26"/>
-      <c r="N5" s="26"/>
-      <c r="O5" s="26"/>
-      <c r="P5" s="26"/>
-      <c r="Q5" s="27"/>
-      <c r="R5" s="27"/>
-      <c r="S5" s="27"/>
-      <c r="T5" s="27"/>
-      <c r="U5" s="28"/>
+      <c r="A5" s="31"/>
+      <c r="B5" s="31"/>
+      <c r="C5" s="31"/>
+      <c r="D5" s="31"/>
+      <c r="E5" s="31"/>
+      <c r="F5" s="31"/>
+      <c r="G5" s="31"/>
+      <c r="H5" s="31"/>
+      <c r="I5" s="31"/>
+      <c r="J5" s="31"/>
+      <c r="K5" s="28"/>
+      <c r="L5" s="28"/>
+      <c r="M5" s="28"/>
+      <c r="N5" s="28"/>
+      <c r="O5" s="28"/>
+      <c r="P5" s="28"/>
+      <c r="Q5" s="29"/>
+      <c r="R5" s="29"/>
+      <c r="S5" s="29"/>
+      <c r="T5" s="29"/>
+      <c r="U5" s="30"/>
     </row>
     <row r="6" ht="15" customHeight="1" spans="1:21">
-      <c r="A6" s="29"/>
-      <c r="B6" s="29"/>
-      <c r="C6" s="29"/>
-      <c r="D6" s="29"/>
-      <c r="E6" s="29"/>
-      <c r="F6" s="29"/>
-      <c r="G6" s="29"/>
-      <c r="H6" s="29"/>
-      <c r="I6" s="29"/>
-      <c r="J6" s="29"/>
-      <c r="K6" s="26"/>
-      <c r="L6" s="26"/>
-      <c r="M6" s="26"/>
-      <c r="N6" s="26"/>
-      <c r="O6" s="26"/>
-      <c r="P6" s="26"/>
-      <c r="Q6" s="27"/>
-      <c r="R6" s="27"/>
-      <c r="S6" s="27"/>
-      <c r="T6" s="27"/>
-      <c r="U6" s="28"/>
+      <c r="A6" s="31"/>
+      <c r="B6" s="31"/>
+      <c r="C6" s="31"/>
+      <c r="D6" s="31"/>
+      <c r="E6" s="31"/>
+      <c r="F6" s="31"/>
+      <c r="G6" s="31"/>
+      <c r="H6" s="31"/>
+      <c r="I6" s="31"/>
+      <c r="J6" s="31"/>
+      <c r="K6" s="28"/>
+      <c r="L6" s="28"/>
+      <c r="M6" s="28"/>
+      <c r="N6" s="28"/>
+      <c r="O6" s="28"/>
+      <c r="P6" s="28"/>
+      <c r="Q6" s="29"/>
+      <c r="R6" s="29"/>
+      <c r="S6" s="29"/>
+      <c r="T6" s="29"/>
+      <c r="U6" s="30"/>
     </row>
     <row r="7" ht="15" customHeight="1" spans="1:21">
-      <c r="A7" s="30"/>
-      <c r="B7" s="26"/>
-      <c r="C7" s="26"/>
-      <c r="D7" s="26"/>
-      <c r="E7" s="26"/>
-      <c r="F7" s="26"/>
-      <c r="G7" s="26"/>
-      <c r="H7" s="26"/>
-      <c r="I7" s="26"/>
-      <c r="J7" s="26"/>
-      <c r="K7" s="26"/>
-      <c r="L7" s="26"/>
-      <c r="M7" s="26"/>
-      <c r="N7" s="26"/>
-      <c r="O7" s="26"/>
-      <c r="P7" s="26"/>
-      <c r="Q7" s="27"/>
-      <c r="R7" s="27"/>
-      <c r="S7" s="27"/>
-      <c r="T7" s="27"/>
-      <c r="U7" s="28"/>
+      <c r="A7" s="32"/>
+      <c r="B7" s="28"/>
+      <c r="C7" s="28"/>
+      <c r="D7" s="28"/>
+      <c r="E7" s="28"/>
+      <c r="F7" s="28"/>
+      <c r="G7" s="28"/>
+      <c r="H7" s="28"/>
+      <c r="I7" s="28"/>
+      <c r="J7" s="28"/>
+      <c r="K7" s="28"/>
+      <c r="L7" s="28"/>
+      <c r="M7" s="28"/>
+      <c r="N7" s="28"/>
+      <c r="O7" s="28"/>
+      <c r="P7" s="28"/>
+      <c r="Q7" s="29"/>
+      <c r="R7" s="29"/>
+      <c r="S7" s="29"/>
+      <c r="T7" s="29"/>
+      <c r="U7" s="30"/>
     </row>
     <row r="8" ht="15" customHeight="1" spans="1:21">
-      <c r="A8" s="31" t="s">
+      <c r="A8" s="33" t="s">
         <v>2</v>
       </c>
-      <c r="B8" s="31"/>
-      <c r="C8" s="31"/>
-      <c r="D8" s="31"/>
-      <c r="E8" s="31"/>
-      <c r="F8" s="31"/>
-      <c r="G8" s="31"/>
-      <c r="H8" s="31"/>
-      <c r="I8" s="31"/>
-      <c r="J8" s="31"/>
-      <c r="K8" s="31"/>
-      <c r="L8" s="31"/>
-      <c r="M8" s="31"/>
-      <c r="N8" s="26"/>
-      <c r="O8" s="26"/>
-      <c r="P8" s="26"/>
-      <c r="Q8" s="27"/>
-      <c r="R8" s="27"/>
-      <c r="S8" s="27"/>
-      <c r="T8" s="27"/>
-      <c r="U8" s="28"/>
+      <c r="B8" s="33"/>
+      <c r="C8" s="33"/>
+      <c r="D8" s="33"/>
+      <c r="E8" s="33"/>
+      <c r="F8" s="33"/>
+      <c r="G8" s="33"/>
+      <c r="H8" s="33"/>
+      <c r="I8" s="33"/>
+      <c r="J8" s="33"/>
+      <c r="K8" s="33"/>
+      <c r="L8" s="33"/>
+      <c r="M8" s="33"/>
+      <c r="N8" s="33"/>
+      <c r="O8" s="28"/>
+      <c r="P8" s="28"/>
+      <c r="Q8" s="29"/>
+      <c r="R8" s="29"/>
+      <c r="S8" s="29"/>
+      <c r="T8" s="29"/>
+      <c r="U8" s="30"/>
     </row>
     <row r="9" ht="15" customHeight="1" spans="1:21">
-      <c r="A9" s="31" t="s">
+      <c r="A9" s="34" t="s">
         <v>3</v>
       </c>
-      <c r="B9" s="31" t="s">
+      <c r="B9" s="34" t="s">
         <v>4</v>
       </c>
-      <c r="C9" s="31"/>
-      <c r="D9" s="31"/>
-      <c r="E9" s="31" t="s">
+      <c r="C9" s="34"/>
+      <c r="D9" s="34"/>
+      <c r="E9" s="34" t="s">
         <v>5</v>
       </c>
-      <c r="F9" s="31"/>
-      <c r="G9" s="31" t="s">
+      <c r="F9" s="34"/>
+      <c r="G9" s="34" t="s">
         <v>6</v>
       </c>
-      <c r="H9" s="31"/>
-      <c r="I9" s="31" t="s">
+      <c r="H9" s="34"/>
+      <c r="I9" s="34" t="s">
         <v>7</v>
       </c>
-      <c r="J9" s="31"/>
-      <c r="K9" s="31" t="s">
+      <c r="J9" s="34"/>
+      <c r="K9" s="34" t="s">
         <v>8</v>
       </c>
-      <c r="L9" s="31" t="s">
+      <c r="L9" s="33" t="s">
         <v>9</v>
       </c>
-      <c r="M9" s="31"/>
-      <c r="N9" s="26"/>
-      <c r="O9" s="26"/>
-      <c r="P9" s="26"/>
-      <c r="Q9" s="27"/>
-      <c r="R9" s="27"/>
-      <c r="S9" s="27"/>
-      <c r="T9" s="27"/>
-      <c r="U9" s="28"/>
-    </row>
-    <row r="10" ht="15" customHeight="1" spans="1:21">
-      <c r="A10" s="31"/>
-      <c r="B10" s="31" t="s">
+      <c r="M9" s="33"/>
+      <c r="N9" s="33"/>
+      <c r="O9" s="28"/>
+      <c r="P9" s="28"/>
+      <c r="Q9" s="29"/>
+      <c r="R9" s="29"/>
+      <c r="S9" s="29"/>
+      <c r="T9" s="29"/>
+      <c r="U9" s="30"/>
+    </row>
+    <row r="10" spans="1:21">
+      <c r="A10" s="34"/>
+      <c r="B10" s="34" t="s">
         <v>10</v>
       </c>
-      <c r="C10" s="31"/>
-      <c r="D10" s="31"/>
-      <c r="E10" s="31" t="s">
+      <c r="C10" s="34"/>
+      <c r="D10" s="34"/>
+      <c r="E10" s="34" t="s">
         <v>11</v>
       </c>
-      <c r="F10" s="31"/>
-      <c r="G10" s="32" t="s">
+      <c r="F10" s="34"/>
+      <c r="G10" s="35" t="s">
         <v>12</v>
       </c>
-      <c r="H10" s="32"/>
-      <c r="I10" s="33" t="s">
+      <c r="H10" s="35"/>
+      <c r="I10" s="34" t="s">
         <v>13</v>
       </c>
       <c r="J10" s="34"/>
-      <c r="K10" s="31" t="s">
+      <c r="K10" s="34" t="s">
         <v>14</v>
       </c>
-      <c r="L10" s="32" t="s">
+      <c r="L10" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="M10" s="32"/>
-      <c r="N10" s="26"/>
-      <c r="O10" s="26"/>
-      <c r="P10" s="26"/>
-      <c r="Q10" s="27"/>
-      <c r="R10" s="27"/>
-      <c r="S10" s="27"/>
-      <c r="T10" s="27"/>
-      <c r="U10" s="28"/>
+      <c r="M10" s="36"/>
+      <c r="N10" s="36"/>
+      <c r="O10" s="28"/>
+      <c r="P10" s="28"/>
+      <c r="Q10" s="29"/>
+      <c r="R10" s="29"/>
+      <c r="S10" s="29"/>
+      <c r="T10" s="29"/>
+      <c r="U10" s="30"/>
     </row>
     <row r="11" ht="15" customHeight="1" spans="1:21">
-      <c r="A11" s="30"/>
-      <c r="B11" s="26"/>
-      <c r="C11" s="26"/>
-      <c r="D11" s="26"/>
-      <c r="E11" s="26"/>
-      <c r="F11" s="26"/>
-      <c r="G11" s="26"/>
-      <c r="H11" s="26"/>
-      <c r="I11" s="26"/>
-      <c r="J11" s="26"/>
-      <c r="K11" s="26"/>
-      <c r="L11" s="26"/>
-      <c r="M11" s="26"/>
-      <c r="N11" s="26"/>
-      <c r="O11" s="26"/>
-      <c r="P11" s="26"/>
-      <c r="Q11" s="27"/>
-      <c r="R11" s="27"/>
-      <c r="S11" s="27"/>
-      <c r="T11" s="27"/>
-      <c r="U11" s="28"/>
+      <c r="A11" s="32"/>
+      <c r="B11" s="28"/>
+      <c r="C11" s="28"/>
+      <c r="D11" s="28"/>
+      <c r="E11" s="28"/>
+      <c r="F11" s="28"/>
+      <c r="G11" s="28"/>
+      <c r="H11" s="28"/>
+      <c r="I11" s="28"/>
+      <c r="J11" s="28"/>
+      <c r="K11" s="28"/>
+      <c r="L11" s="28"/>
+      <c r="M11" s="28"/>
+      <c r="N11" s="28"/>
+      <c r="O11" s="28"/>
+      <c r="P11" s="28"/>
+      <c r="Q11" s="29"/>
+      <c r="R11" s="29"/>
+      <c r="S11" s="29"/>
+      <c r="T11" s="29"/>
+      <c r="U11" s="30"/>
     </row>
     <row r="12" ht="15" customHeight="1" spans="1:21">
-      <c r="A12" s="30"/>
-      <c r="B12" s="26"/>
-      <c r="C12" s="26"/>
-      <c r="D12" s="26"/>
-      <c r="E12" s="26"/>
-      <c r="F12" s="26"/>
-      <c r="G12" s="26"/>
-      <c r="H12" s="26"/>
-      <c r="I12" s="26"/>
-      <c r="J12" s="26"/>
-      <c r="K12" s="26"/>
-      <c r="L12" s="26"/>
-      <c r="M12" s="26"/>
-      <c r="N12" s="26"/>
-      <c r="O12" s="26"/>
-      <c r="P12" s="26"/>
-      <c r="Q12" s="27"/>
-      <c r="R12" s="27"/>
-      <c r="S12" s="27"/>
-      <c r="T12" s="27"/>
-      <c r="U12" s="28"/>
+      <c r="A12" s="32"/>
+      <c r="B12" s="28"/>
+      <c r="C12" s="28"/>
+      <c r="D12" s="28"/>
+      <c r="E12" s="28"/>
+      <c r="F12" s="28"/>
+      <c r="G12" s="28"/>
+      <c r="H12" s="28"/>
+      <c r="I12" s="28"/>
+      <c r="J12" s="28"/>
+      <c r="K12" s="28"/>
+      <c r="L12" s="28"/>
+      <c r="M12" s="28"/>
+      <c r="N12" s="28"/>
+      <c r="O12" s="28"/>
+      <c r="P12" s="28"/>
+      <c r="Q12" s="29"/>
+      <c r="R12" s="29"/>
+      <c r="S12" s="29"/>
+      <c r="T12" s="29"/>
+      <c r="U12" s="30"/>
     </row>
     <row r="13" ht="15" customHeight="1" spans="1:21">
-      <c r="A13" s="32" t="s">
+      <c r="A13" s="35" t="s">
         <v>16</v>
       </c>
-      <c r="B13" s="32"/>
-      <c r="C13" s="31" t="s">
+      <c r="B13" s="35"/>
+      <c r="C13" s="34" t="s">
         <v>17</v>
       </c>
-      <c r="D13" s="31"/>
-      <c r="E13" s="31"/>
-      <c r="F13" s="31"/>
-      <c r="G13" s="31"/>
-      <c r="H13" s="31"/>
-      <c r="I13" s="31"/>
-      <c r="J13" s="31"/>
-      <c r="K13" s="31"/>
-      <c r="L13" s="31"/>
-      <c r="M13" s="31"/>
-      <c r="N13" s="31"/>
-      <c r="O13" s="31"/>
-      <c r="P13" s="31"/>
-      <c r="Q13" s="31"/>
-      <c r="R13" s="31"/>
-      <c r="S13" s="31"/>
-      <c r="T13" s="31"/>
-      <c r="U13" s="31"/>
+      <c r="D13" s="34"/>
+      <c r="E13" s="34"/>
+      <c r="F13" s="34"/>
+      <c r="G13" s="34"/>
+      <c r="H13" s="34"/>
+      <c r="I13" s="34"/>
+      <c r="J13" s="34"/>
+      <c r="K13" s="34"/>
+      <c r="L13" s="34"/>
+      <c r="M13" s="34"/>
+      <c r="N13" s="34"/>
+      <c r="O13" s="34"/>
+      <c r="P13" s="34"/>
+      <c r="Q13" s="34"/>
+      <c r="R13" s="34"/>
+      <c r="S13" s="34"/>
+      <c r="T13" s="34"/>
+      <c r="U13" s="34"/>
     </row>
     <row r="14" ht="15" customHeight="1" spans="1:21">
-      <c r="A14" s="32"/>
-      <c r="B14" s="32"/>
-      <c r="C14" s="31" t="s">
+      <c r="A14" s="35"/>
+      <c r="B14" s="35"/>
+      <c r="C14" s="34" t="s">
         <v>18</v>
       </c>
-      <c r="D14" s="31"/>
-      <c r="E14" s="31"/>
-      <c r="F14" s="31" t="s">
+      <c r="D14" s="34"/>
+      <c r="E14" s="34"/>
+      <c r="F14" s="34" t="s">
         <v>19</v>
       </c>
-      <c r="G14" s="31"/>
-      <c r="H14" s="31"/>
-      <c r="I14" s="31" t="s">
+      <c r="G14" s="34"/>
+      <c r="H14" s="34"/>
+      <c r="I14" s="34" t="s">
         <v>20</v>
       </c>
-      <c r="J14" s="31"/>
-      <c r="K14" s="31"/>
-      <c r="L14" s="31" t="s">
+      <c r="J14" s="34"/>
+      <c r="K14" s="34"/>
+      <c r="L14" s="34" t="s">
         <v>21</v>
       </c>
-      <c r="M14" s="31"/>
-      <c r="N14" s="31"/>
-      <c r="O14" s="31" t="s">
+      <c r="M14" s="34"/>
+      <c r="N14" s="34"/>
+      <c r="O14" s="34" t="s">
         <v>22</v>
       </c>
-      <c r="P14" s="31"/>
-      <c r="Q14" s="31"/>
-      <c r="R14" s="31" t="s">
+      <c r="P14" s="34"/>
+      <c r="Q14" s="34"/>
+      <c r="R14" s="34" t="s">
         <v>23</v>
       </c>
-      <c r="S14" s="31"/>
-      <c r="T14" s="35" t="s">
+      <c r="S14" s="34"/>
+      <c r="T14" s="37" t="s">
         <v>24</v>
       </c>
-      <c r="U14" s="35" t="s">
+      <c r="U14" s="37" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1" spans="1:21">
-      <c r="A15" s="32"/>
-      <c r="B15" s="32"/>
-      <c r="C15" s="36" t="s">
+      <c r="A15" s="35"/>
+      <c r="B15" s="35"/>
+      <c r="C15" s="38" t="s">
         <v>26</v>
       </c>
-      <c r="D15" s="36"/>
-      <c r="E15" s="36"/>
-      <c r="F15" s="36" t="s">
+      <c r="D15" s="38"/>
+      <c r="E15" s="38"/>
+      <c r="F15" s="38" t="s">
         <v>27</v>
       </c>
-      <c r="G15" s="37"/>
-      <c r="H15" s="38"/>
-      <c r="I15" s="35" t="s">
+      <c r="G15" s="39"/>
+      <c r="H15" s="20"/>
+      <c r="I15" s="37" t="s">
         <v>28</v>
       </c>
-      <c r="J15" s="35"/>
-      <c r="K15" s="38"/>
-      <c r="L15" s="35" t="s">
+      <c r="J15" s="37"/>
+      <c r="K15" s="20"/>
+      <c r="L15" s="37" t="s">
         <v>29</v>
       </c>
-      <c r="M15" s="35"/>
-      <c r="N15" s="38"/>
-      <c r="O15" s="35" t="s">
+      <c r="M15" s="37"/>
+      <c r="N15" s="20"/>
+      <c r="O15" s="37" t="s">
         <v>30</v>
       </c>
-      <c r="P15" s="35"/>
-      <c r="Q15" s="38"/>
-      <c r="R15" s="35" t="s">
+      <c r="P15" s="37"/>
+      <c r="Q15" s="20"/>
+      <c r="R15" s="37" t="s">
         <v>31</v>
       </c>
-      <c r="S15" s="35"/>
-      <c r="T15" s="35" t="s">
+      <c r="S15" s="37"/>
+      <c r="T15" s="37" t="s">
         <v>18</v>
       </c>
-      <c r="U15" s="35" t="s">
+      <c r="U15" s="37" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1" spans="1:21">
-      <c r="A16" s="32"/>
-      <c r="B16" s="32"/>
-      <c r="C16" s="29" t="s">
+      <c r="A16" s="35"/>
+      <c r="B16" s="35"/>
+      <c r="C16" s="31" t="s">
         <v>33</v>
       </c>
-      <c r="D16" s="29"/>
-      <c r="E16" s="29"/>
-      <c r="F16" s="29"/>
-      <c r="G16" s="29"/>
-      <c r="H16" s="29"/>
-      <c r="I16" s="29"/>
-      <c r="J16" s="29"/>
-      <c r="K16" s="29"/>
-      <c r="L16" s="29"/>
-      <c r="M16" s="29"/>
-      <c r="N16" s="29"/>
-      <c r="O16" s="29"/>
-      <c r="P16" s="29"/>
-      <c r="Q16" s="29"/>
-      <c r="R16" s="29"/>
-      <c r="S16" s="29"/>
-      <c r="T16" s="29"/>
-      <c r="U16" s="29"/>
+      <c r="D16" s="31"/>
+      <c r="E16" s="31"/>
+      <c r="F16" s="31"/>
+      <c r="G16" s="31"/>
+      <c r="H16" s="31"/>
+      <c r="I16" s="31"/>
+      <c r="J16" s="31"/>
+      <c r="K16" s="31"/>
+      <c r="L16" s="31"/>
+      <c r="M16" s="31"/>
+      <c r="N16" s="31"/>
+      <c r="O16" s="31"/>
+      <c r="P16" s="31"/>
+      <c r="Q16" s="31"/>
+      <c r="R16" s="31"/>
+      <c r="S16" s="31"/>
+      <c r="T16" s="31"/>
+      <c r="U16" s="31"/>
     </row>
     <row r="17" ht="15" customHeight="1" spans="1:21">
-      <c r="A17" s="32"/>
-      <c r="B17" s="32"/>
-      <c r="C17" s="29"/>
-      <c r="D17" s="29"/>
-      <c r="E17" s="29"/>
-      <c r="F17" s="29"/>
-      <c r="G17" s="29"/>
-      <c r="H17" s="29"/>
-      <c r="I17" s="29"/>
-      <c r="J17" s="29"/>
-      <c r="K17" s="29"/>
-      <c r="L17" s="29"/>
-      <c r="M17" s="29"/>
-      <c r="N17" s="29"/>
-      <c r="O17" s="29"/>
-      <c r="P17" s="29"/>
-      <c r="Q17" s="29"/>
-      <c r="R17" s="29"/>
-      <c r="S17" s="29"/>
-      <c r="T17" s="29"/>
-      <c r="U17" s="29"/>
+      <c r="A17" s="35"/>
+      <c r="B17" s="35"/>
+      <c r="C17" s="31"/>
+      <c r="D17" s="31"/>
+      <c r="E17" s="31"/>
+      <c r="F17" s="31"/>
+      <c r="G17" s="31"/>
+      <c r="H17" s="31"/>
+      <c r="I17" s="31"/>
+      <c r="J17" s="31"/>
+      <c r="K17" s="31"/>
+      <c r="L17" s="31"/>
+      <c r="M17" s="31"/>
+      <c r="N17" s="31"/>
+      <c r="O17" s="31"/>
+      <c r="P17" s="31"/>
+      <c r="Q17" s="31"/>
+      <c r="R17" s="31"/>
+      <c r="S17" s="31"/>
+      <c r="T17" s="31"/>
+      <c r="U17" s="31"/>
     </row>
     <row r="18" ht="15" customHeight="1" spans="1:21">
-      <c r="A18" s="32"/>
-      <c r="B18" s="32"/>
-      <c r="C18" s="26"/>
-      <c r="D18" s="26"/>
-      <c r="E18" s="26"/>
-      <c r="F18" s="26"/>
-      <c r="G18" s="26"/>
-      <c r="H18" s="26"/>
-      <c r="I18" s="26"/>
-      <c r="J18" s="26"/>
-      <c r="K18" s="26"/>
-      <c r="L18" s="26"/>
-      <c r="M18" s="26"/>
-      <c r="N18" s="26"/>
-      <c r="O18" s="26"/>
-      <c r="P18" s="26"/>
-      <c r="Q18" s="27"/>
-      <c r="R18" s="27"/>
-      <c r="S18" s="27"/>
-      <c r="T18" s="27"/>
-      <c r="U18" s="28"/>
+      <c r="A18" s="35"/>
+      <c r="B18" s="35"/>
+      <c r="C18" s="28"/>
+      <c r="D18" s="28"/>
+      <c r="E18" s="28"/>
+      <c r="F18" s="28"/>
+      <c r="G18" s="28"/>
+      <c r="H18" s="28"/>
+      <c r="I18" s="28"/>
+      <c r="J18" s="28"/>
+      <c r="K18" s="28"/>
+      <c r="L18" s="28"/>
+      <c r="M18" s="28"/>
+      <c r="N18" s="28"/>
+      <c r="O18" s="28"/>
+      <c r="P18" s="28"/>
+      <c r="Q18" s="29"/>
+      <c r="R18" s="29"/>
+      <c r="S18" s="29"/>
+      <c r="T18" s="29"/>
+      <c r="U18" s="30"/>
     </row>
     <row r="19" ht="15" customHeight="1" spans="1:21">
-      <c r="A19" s="32"/>
-      <c r="B19" s="32"/>
-      <c r="C19" s="34" t="s">
+      <c r="A19" s="35"/>
+      <c r="B19" s="35"/>
+      <c r="C19" s="40" t="s">
         <v>34</v>
       </c>
-      <c r="D19" s="31"/>
-      <c r="E19" s="31"/>
-      <c r="F19" s="31"/>
-      <c r="G19" s="31"/>
-      <c r="H19" s="31"/>
-      <c r="I19" s="31"/>
-      <c r="J19" s="31"/>
-      <c r="K19" s="31"/>
-      <c r="L19" s="31"/>
-      <c r="M19" s="26"/>
-      <c r="N19" s="26"/>
-      <c r="O19" s="26"/>
-      <c r="P19" s="26"/>
-      <c r="Q19" s="27"/>
-      <c r="R19" s="27"/>
-      <c r="S19" s="27"/>
-      <c r="T19" s="27"/>
-      <c r="U19" s="28"/>
+      <c r="D19" s="34"/>
+      <c r="E19" s="34"/>
+      <c r="F19" s="34"/>
+      <c r="G19" s="34"/>
+      <c r="H19" s="34"/>
+      <c r="I19" s="34"/>
+      <c r="J19" s="34"/>
+      <c r="K19" s="34"/>
+      <c r="L19" s="34"/>
+      <c r="M19" s="28"/>
+      <c r="N19" s="28"/>
+      <c r="O19" s="28"/>
+      <c r="P19" s="28"/>
+      <c r="Q19" s="29"/>
+      <c r="R19" s="29"/>
+      <c r="S19" s="29"/>
+      <c r="T19" s="29"/>
+      <c r="U19" s="30"/>
     </row>
     <row r="20" ht="15" customHeight="1" spans="1:21">
-      <c r="A20" s="32"/>
-      <c r="B20" s="32"/>
-      <c r="C20" s="34" t="s">
+      <c r="A20" s="35"/>
+      <c r="B20" s="35"/>
+      <c r="C20" s="40" t="s">
         <v>34</v>
       </c>
-      <c r="D20" s="31"/>
-      <c r="E20" s="31" t="s">
+      <c r="D20" s="34"/>
+      <c r="E20" s="34" t="s">
         <v>35</v>
       </c>
-      <c r="F20" s="31"/>
-      <c r="G20" s="31"/>
-      <c r="H20" s="31"/>
-      <c r="I20" s="31"/>
-      <c r="J20" s="31"/>
-      <c r="K20" s="31" t="s">
+      <c r="F20" s="34"/>
+      <c r="G20" s="34"/>
+      <c r="H20" s="34"/>
+      <c r="I20" s="34"/>
+      <c r="J20" s="34"/>
+      <c r="K20" s="34" t="s">
         <v>36</v>
       </c>
-      <c r="L20" s="31"/>
-      <c r="M20" s="26"/>
-      <c r="N20" s="26"/>
-      <c r="O20" s="26"/>
-      <c r="P20" s="26"/>
-      <c r="Q20" s="27"/>
-      <c r="R20" s="27"/>
-      <c r="S20" s="27"/>
-      <c r="T20" s="27"/>
-      <c r="U20" s="28"/>
+      <c r="L20" s="34"/>
+      <c r="M20" s="28"/>
+      <c r="N20" s="28"/>
+      <c r="O20" s="28"/>
+      <c r="P20" s="28"/>
+      <c r="Q20" s="29"/>
+      <c r="R20" s="29"/>
+      <c r="S20" s="29"/>
+      <c r="T20" s="29"/>
+      <c r="U20" s="30"/>
     </row>
     <row r="21" ht="15" customHeight="1" spans="1:21">
-      <c r="A21" s="32"/>
-      <c r="B21" s="32"/>
-      <c r="C21" s="34" t="s">
+      <c r="A21" s="35"/>
+      <c r="B21" s="35"/>
+      <c r="C21" s="40" t="s">
         <v>37</v>
       </c>
-      <c r="D21" s="31"/>
-      <c r="E21" s="39" t="s">
+      <c r="D21" s="34"/>
+      <c r="E21" s="41" t="s">
         <v>38</v>
       </c>
-      <c r="F21" s="40"/>
-      <c r="G21" s="40"/>
-      <c r="H21" s="40"/>
-      <c r="I21" s="40"/>
-      <c r="J21" s="41"/>
-      <c r="K21" s="31" t="s">
+      <c r="F21" s="42"/>
+      <c r="G21" s="42"/>
+      <c r="H21" s="42"/>
+      <c r="I21" s="42"/>
+      <c r="J21" s="40"/>
+      <c r="K21" s="34" t="s">
         <v>39</v>
       </c>
-      <c r="L21" s="31"/>
-      <c r="M21" s="26"/>
-      <c r="N21" s="26"/>
-      <c r="O21" s="26"/>
-      <c r="P21" s="26"/>
-      <c r="Q21" s="27"/>
-      <c r="R21" s="27"/>
-      <c r="S21" s="27"/>
-      <c r="T21" s="27"/>
-      <c r="U21" s="28"/>
+      <c r="L21" s="34"/>
+      <c r="M21" s="28"/>
+      <c r="N21" s="28"/>
+      <c r="O21" s="28"/>
+      <c r="P21" s="28"/>
+      <c r="Q21" s="29"/>
+      <c r="R21" s="29"/>
+      <c r="S21" s="29"/>
+      <c r="T21" s="29"/>
+      <c r="U21" s="30"/>
     </row>
     <row r="22" ht="15" customHeight="1" spans="1:21">
-      <c r="A22" s="32"/>
-      <c r="B22" s="32"/>
-      <c r="C22" s="34" t="s">
+      <c r="A22" s="35"/>
+      <c r="B22" s="35"/>
+      <c r="C22" s="40" t="s">
         <v>40</v>
       </c>
-      <c r="D22" s="31"/>
-      <c r="E22" s="31" t="s">
+      <c r="D22" s="34"/>
+      <c r="E22" s="34" t="s">
         <v>41</v>
       </c>
-      <c r="F22" s="31"/>
-      <c r="G22" s="31"/>
-      <c r="H22" s="31"/>
-      <c r="I22" s="31"/>
-      <c r="J22" s="31"/>
-      <c r="K22" s="31" t="s">
+      <c r="F22" s="34"/>
+      <c r="G22" s="34"/>
+      <c r="H22" s="34"/>
+      <c r="I22" s="34"/>
+      <c r="J22" s="34"/>
+      <c r="K22" s="34" t="s">
         <v>39</v>
       </c>
-      <c r="L22" s="31"/>
-      <c r="M22" s="26"/>
-      <c r="N22" s="26"/>
-      <c r="O22" s="26"/>
-      <c r="P22" s="26"/>
-      <c r="Q22" s="27"/>
-      <c r="R22" s="27"/>
-      <c r="S22" s="27"/>
-      <c r="T22" s="27"/>
-      <c r="U22" s="28"/>
+      <c r="L22" s="34"/>
+      <c r="M22" s="28"/>
+      <c r="N22" s="28"/>
+      <c r="O22" s="28"/>
+      <c r="P22" s="28"/>
+      <c r="Q22" s="29"/>
+      <c r="R22" s="29"/>
+      <c r="S22" s="29"/>
+      <c r="T22" s="29"/>
+      <c r="U22" s="30"/>
     </row>
     <row r="23" ht="15" customHeight="1" spans="1:21">
-      <c r="A23" s="32"/>
-      <c r="B23" s="32"/>
-      <c r="C23" s="34" t="s">
+      <c r="A23" s="35"/>
+      <c r="B23" s="35"/>
+      <c r="C23" s="40" t="s">
         <v>42</v>
       </c>
-      <c r="D23" s="31"/>
-      <c r="E23" s="31" t="s">
+      <c r="D23" s="34"/>
+      <c r="E23" s="34" t="s">
         <v>43</v>
       </c>
-      <c r="F23" s="31"/>
-      <c r="G23" s="31"/>
-      <c r="H23" s="31"/>
-      <c r="I23" s="31"/>
-      <c r="J23" s="31"/>
-      <c r="K23" s="31" t="s">
+      <c r="F23" s="34"/>
+      <c r="G23" s="34"/>
+      <c r="H23" s="34"/>
+      <c r="I23" s="34"/>
+      <c r="J23" s="34"/>
+      <c r="K23" s="34" t="s">
         <v>39</v>
       </c>
-      <c r="L23" s="31"/>
-      <c r="M23" s="26"/>
-      <c r="N23" s="26"/>
-      <c r="O23" s="26"/>
-      <c r="P23" s="26"/>
-      <c r="Q23" s="27"/>
-      <c r="R23" s="27"/>
-      <c r="S23" s="27"/>
-      <c r="T23" s="27"/>
-      <c r="U23" s="28"/>
+      <c r="L23" s="34"/>
+      <c r="M23" s="28"/>
+      <c r="N23" s="28"/>
+      <c r="O23" s="28"/>
+      <c r="P23" s="28"/>
+      <c r="Q23" s="29"/>
+      <c r="R23" s="29"/>
+      <c r="S23" s="29"/>
+      <c r="T23" s="29"/>
+      <c r="U23" s="30"/>
     </row>
     <row r="24" ht="15" customHeight="1" spans="1:21">
-      <c r="A24" s="32"/>
-      <c r="B24" s="32"/>
+      <c r="A24" s="35"/>
+      <c r="B24" s="35"/>
       <c r="C24" s="9"/>
       <c r="D24" s="9"/>
       <c r="E24" s="9"/>
@@ -2350,205 +2384,205 @@
       <c r="J24" s="9"/>
       <c r="K24" s="9"/>
       <c r="L24" s="9"/>
-      <c r="M24" s="26"/>
-      <c r="N24" s="26"/>
-      <c r="O24" s="26"/>
-      <c r="P24" s="26"/>
-      <c r="Q24" s="27"/>
-      <c r="R24" s="27"/>
-      <c r="S24" s="27"/>
-      <c r="T24" s="27"/>
-      <c r="U24" s="28"/>
+      <c r="M24" s="28"/>
+      <c r="N24" s="28"/>
+      <c r="O24" s="28"/>
+      <c r="P24" s="28"/>
+      <c r="Q24" s="29"/>
+      <c r="R24" s="29"/>
+      <c r="S24" s="29"/>
+      <c r="T24" s="29"/>
+      <c r="U24" s="30"/>
     </row>
     <row r="25" ht="15" customHeight="1" spans="1:21">
-      <c r="A25" s="32"/>
-      <c r="B25" s="32"/>
-      <c r="C25" s="36" t="s">
+      <c r="A25" s="35"/>
+      <c r="B25" s="35"/>
+      <c r="C25" s="38" t="s">
         <v>44</v>
       </c>
-      <c r="D25" s="36"/>
-      <c r="E25" s="36"/>
-      <c r="F25" s="36"/>
-      <c r="G25" s="42"/>
-      <c r="H25" s="42"/>
-      <c r="I25" s="42"/>
-      <c r="J25" s="42"/>
-      <c r="K25" s="42"/>
-      <c r="L25" s="42"/>
-      <c r="M25" s="42"/>
-      <c r="N25" s="42"/>
-      <c r="O25" s="26"/>
-      <c r="P25" s="26"/>
-      <c r="Q25" s="27"/>
-      <c r="R25" s="27"/>
-      <c r="S25" s="27"/>
-      <c r="T25" s="27"/>
-      <c r="U25" s="28"/>
+      <c r="D25" s="38"/>
+      <c r="E25" s="38"/>
+      <c r="F25" s="38"/>
+      <c r="G25" s="43"/>
+      <c r="H25" s="43"/>
+      <c r="I25" s="43"/>
+      <c r="J25" s="43"/>
+      <c r="K25" s="43"/>
+      <c r="L25" s="43"/>
+      <c r="M25" s="43"/>
+      <c r="N25" s="43"/>
+      <c r="O25" s="28"/>
+      <c r="P25" s="28"/>
+      <c r="Q25" s="29"/>
+      <c r="R25" s="29"/>
+      <c r="S25" s="29"/>
+      <c r="T25" s="29"/>
+      <c r="U25" s="30"/>
     </row>
     <row r="26" ht="15" customHeight="1" spans="1:21">
-      <c r="A26" s="32"/>
-      <c r="B26" s="32"/>
-      <c r="C26" s="31" t="s">
+      <c r="A26" s="35"/>
+      <c r="B26" s="35"/>
+      <c r="C26" s="34" t="s">
         <v>45</v>
       </c>
-      <c r="D26" s="31"/>
-      <c r="E26" s="31"/>
-      <c r="F26" s="31"/>
-      <c r="G26" s="43"/>
-      <c r="H26" s="43"/>
-      <c r="I26" s="43"/>
-      <c r="J26" s="43"/>
-      <c r="K26" s="43"/>
-      <c r="L26" s="43"/>
-      <c r="M26" s="43"/>
-      <c r="N26" s="43"/>
-      <c r="O26" s="26"/>
-      <c r="P26" s="26"/>
-      <c r="Q26" s="27"/>
-      <c r="R26" s="27"/>
-      <c r="S26" s="27"/>
-      <c r="T26" s="27"/>
-      <c r="U26" s="28"/>
+      <c r="D26" s="34"/>
+      <c r="E26" s="34"/>
+      <c r="F26" s="34"/>
+      <c r="G26" s="44"/>
+      <c r="H26" s="44"/>
+      <c r="I26" s="44"/>
+      <c r="J26" s="44"/>
+      <c r="K26" s="44"/>
+      <c r="L26" s="44"/>
+      <c r="M26" s="44"/>
+      <c r="N26" s="44"/>
+      <c r="O26" s="28"/>
+      <c r="P26" s="28"/>
+      <c r="Q26" s="29"/>
+      <c r="R26" s="29"/>
+      <c r="S26" s="29"/>
+      <c r="T26" s="29"/>
+      <c r="U26" s="30"/>
     </row>
     <row r="27" ht="15" customHeight="1" spans="1:21">
-      <c r="A27" s="32"/>
-      <c r="B27" s="32"/>
-      <c r="C27" s="31" t="s">
+      <c r="A27" s="35"/>
+      <c r="B27" s="35"/>
+      <c r="C27" s="34" t="s">
         <v>46</v>
       </c>
-      <c r="D27" s="31"/>
-      <c r="E27" s="31" t="s">
+      <c r="D27" s="34"/>
+      <c r="E27" s="34" t="s">
         <v>47</v>
       </c>
-      <c r="F27" s="31"/>
-      <c r="G27" s="43"/>
-      <c r="H27" s="43"/>
-      <c r="I27" s="43"/>
-      <c r="J27" s="43"/>
-      <c r="K27" s="43"/>
-      <c r="L27" s="43"/>
-      <c r="M27" s="43"/>
-      <c r="N27" s="43"/>
-      <c r="O27" s="26"/>
-      <c r="P27" s="26"/>
-      <c r="Q27" s="27"/>
-      <c r="R27" s="27"/>
-      <c r="S27" s="27"/>
-      <c r="T27" s="27"/>
-      <c r="U27" s="28"/>
+      <c r="F27" s="34"/>
+      <c r="G27" s="44"/>
+      <c r="H27" s="44"/>
+      <c r="I27" s="44"/>
+      <c r="J27" s="44"/>
+      <c r="K27" s="44"/>
+      <c r="L27" s="44"/>
+      <c r="M27" s="44"/>
+      <c r="N27" s="44"/>
+      <c r="O27" s="28"/>
+      <c r="P27" s="28"/>
+      <c r="Q27" s="29"/>
+      <c r="R27" s="29"/>
+      <c r="S27" s="29"/>
+      <c r="T27" s="29"/>
+      <c r="U27" s="30"/>
     </row>
     <row r="28" ht="15" customHeight="1" spans="1:21">
-      <c r="A28" s="32"/>
-      <c r="B28" s="32"/>
-      <c r="C28" s="44" t="s">
+      <c r="A28" s="35"/>
+      <c r="B28" s="35"/>
+      <c r="C28" s="45" t="s">
         <v>48</v>
       </c>
-      <c r="D28" s="44"/>
-      <c r="E28" s="44" t="s">
+      <c r="D28" s="45"/>
+      <c r="E28" s="45" t="s">
         <v>49</v>
       </c>
-      <c r="F28" s="44"/>
-      <c r="G28" s="43"/>
-      <c r="H28" s="43"/>
-      <c r="I28" s="43"/>
-      <c r="J28" s="43"/>
-      <c r="K28" s="43"/>
-      <c r="L28" s="43"/>
-      <c r="M28" s="43"/>
-      <c r="N28" s="43"/>
-      <c r="O28" s="26"/>
-      <c r="P28" s="26"/>
-      <c r="Q28" s="27"/>
-      <c r="R28" s="27"/>
-      <c r="S28" s="27"/>
-      <c r="T28" s="27"/>
-      <c r="U28" s="28"/>
+      <c r="F28" s="45"/>
+      <c r="G28" s="44"/>
+      <c r="H28" s="44"/>
+      <c r="I28" s="44"/>
+      <c r="J28" s="44"/>
+      <c r="K28" s="44"/>
+      <c r="L28" s="44"/>
+      <c r="M28" s="44"/>
+      <c r="N28" s="44"/>
+      <c r="O28" s="28"/>
+      <c r="P28" s="28"/>
+      <c r="Q28" s="29"/>
+      <c r="R28" s="29"/>
+      <c r="S28" s="29"/>
+      <c r="T28" s="29"/>
+      <c r="U28" s="30"/>
     </row>
     <row r="29" ht="15" customHeight="1" spans="1:21">
-      <c r="A29" s="32"/>
-      <c r="B29" s="32"/>
-      <c r="C29" s="29" t="s">
+      <c r="A29" s="35"/>
+      <c r="B29" s="35"/>
+      <c r="C29" s="31" t="s">
         <v>50</v>
       </c>
-      <c r="D29" s="45"/>
-      <c r="E29" s="45"/>
-      <c r="F29" s="45"/>
-      <c r="G29" s="45"/>
-      <c r="H29" s="45"/>
-      <c r="I29" s="45"/>
-      <c r="J29" s="45"/>
-      <c r="K29" s="26"/>
-      <c r="L29" s="26"/>
-      <c r="M29" s="26"/>
-      <c r="N29" s="26"/>
-      <c r="O29" s="26"/>
-      <c r="P29" s="26"/>
-      <c r="Q29" s="27"/>
-      <c r="R29" s="27"/>
-      <c r="S29" s="27"/>
-      <c r="T29" s="27"/>
-      <c r="U29" s="28"/>
+      <c r="D29" s="46"/>
+      <c r="E29" s="46"/>
+      <c r="F29" s="46"/>
+      <c r="G29" s="46"/>
+      <c r="H29" s="46"/>
+      <c r="I29" s="46"/>
+      <c r="J29" s="46"/>
+      <c r="K29" s="28"/>
+      <c r="L29" s="28"/>
+      <c r="M29" s="28"/>
+      <c r="N29" s="28"/>
+      <c r="O29" s="28"/>
+      <c r="P29" s="28"/>
+      <c r="Q29" s="29"/>
+      <c r="R29" s="29"/>
+      <c r="S29" s="29"/>
+      <c r="T29" s="29"/>
+      <c r="U29" s="30"/>
     </row>
     <row r="30" ht="15" customHeight="1" spans="1:21">
-      <c r="A30" s="32"/>
-      <c r="B30" s="32"/>
-      <c r="C30" s="45"/>
-      <c r="D30" s="45"/>
-      <c r="E30" s="45"/>
-      <c r="F30" s="45"/>
-      <c r="G30" s="45"/>
-      <c r="H30" s="45"/>
-      <c r="I30" s="45"/>
-      <c r="J30" s="45"/>
-      <c r="K30" s="26"/>
-      <c r="L30" s="26"/>
-      <c r="M30" s="26"/>
-      <c r="N30" s="26"/>
-      <c r="O30" s="26"/>
-      <c r="P30" s="26"/>
-      <c r="Q30" s="27"/>
-      <c r="R30" s="27"/>
-      <c r="S30" s="27"/>
-      <c r="T30" s="27"/>
-      <c r="U30" s="28"/>
+      <c r="A30" s="35"/>
+      <c r="B30" s="35"/>
+      <c r="C30" s="46"/>
+      <c r="D30" s="46"/>
+      <c r="E30" s="46"/>
+      <c r="F30" s="46"/>
+      <c r="G30" s="46"/>
+      <c r="H30" s="46"/>
+      <c r="I30" s="46"/>
+      <c r="J30" s="46"/>
+      <c r="K30" s="28"/>
+      <c r="L30" s="28"/>
+      <c r="M30" s="28"/>
+      <c r="N30" s="28"/>
+      <c r="O30" s="28"/>
+      <c r="P30" s="28"/>
+      <c r="Q30" s="29"/>
+      <c r="R30" s="29"/>
+      <c r="S30" s="29"/>
+      <c r="T30" s="29"/>
+      <c r="U30" s="30"/>
     </row>
     <row r="31" ht="15" customHeight="1" spans="1:21">
-      <c r="A31" s="32"/>
-      <c r="B31" s="32"/>
-      <c r="C31" s="45"/>
-      <c r="D31" s="45"/>
-      <c r="E31" s="45"/>
-      <c r="F31" s="45"/>
-      <c r="G31" s="45"/>
-      <c r="H31" s="45"/>
-      <c r="I31" s="45"/>
-      <c r="J31" s="45"/>
-      <c r="K31" s="46"/>
-      <c r="L31" s="46"/>
-      <c r="M31" s="46"/>
-      <c r="N31" s="46"/>
-      <c r="O31" s="46"/>
-      <c r="P31" s="46"/>
-      <c r="Q31" s="46"/>
-      <c r="R31" s="46"/>
-      <c r="S31" s="46"/>
-      <c r="T31" s="46"/>
-      <c r="U31" s="47"/>
+      <c r="A31" s="35"/>
+      <c r="B31" s="35"/>
+      <c r="C31" s="46"/>
+      <c r="D31" s="46"/>
+      <c r="E31" s="46"/>
+      <c r="F31" s="46"/>
+      <c r="G31" s="46"/>
+      <c r="H31" s="46"/>
+      <c r="I31" s="46"/>
+      <c r="J31" s="46"/>
+      <c r="K31" s="47"/>
+      <c r="L31" s="47"/>
+      <c r="M31" s="47"/>
+      <c r="N31" s="47"/>
+      <c r="O31" s="47"/>
+      <c r="P31" s="47"/>
+      <c r="Q31" s="47"/>
+      <c r="R31" s="47"/>
+      <c r="S31" s="47"/>
+      <c r="T31" s="47"/>
+      <c r="U31" s="48"/>
     </row>
   </sheetData>
   <mergeCells count="52">
     <mergeCell ref="A2:J2"/>
-    <mergeCell ref="A8:M8"/>
+    <mergeCell ref="A8:N8"/>
     <mergeCell ref="B9:D9"/>
     <mergeCell ref="E9:F9"/>
     <mergeCell ref="G9:H9"/>
     <mergeCell ref="I9:J9"/>
-    <mergeCell ref="L9:M9"/>
+    <mergeCell ref="L9:N9"/>
     <mergeCell ref="B10:D10"/>
     <mergeCell ref="E10:F10"/>
     <mergeCell ref="G10:H10"/>
     <mergeCell ref="I10:J10"/>
-    <mergeCell ref="L10:M10"/>
+    <mergeCell ref="L10:N10"/>
     <mergeCell ref="C13:U13"/>
     <mergeCell ref="C14:E14"/>
     <mergeCell ref="F14:H14"/>
@@ -2608,31 +2642,31 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" s="19" t="s">
+      <c r="A1" s="21" t="s">
         <v>51</v>
       </c>
-      <c r="B1" s="19"/>
-      <c r="C1" s="19"/>
+      <c r="B1" s="21"/>
+      <c r="C1" s="21"/>
     </row>
     <row r="2" s="1" customFormat="1" spans="1:3">
-      <c r="A2" s="20" t="s">
+      <c r="A2" s="22" t="s">
         <v>52</v>
       </c>
-      <c r="B2" s="20" t="s">
+      <c r="B2" s="22" t="s">
         <v>53</v>
       </c>
-      <c r="C2" s="20" t="s">
+      <c r="C2" s="22" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="3" spans="1:3">
-      <c r="A3" s="20" t="s">
+      <c r="A3" s="22" t="s">
         <v>55</v>
       </c>
-      <c r="B3" s="21" t="s">
+      <c r="B3" s="23" t="s">
         <v>56</v>
       </c>
-      <c r="C3" s="20" t="s">
+      <c r="C3" s="22" t="s">
         <v>57</v>
       </c>
     </row>
@@ -2646,6 +2680,184 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="C8:G26"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelCol="6"/>
+  <cols>
+    <col min="3" max="3" width="13.75" customWidth="1"/>
+    <col min="4" max="4" width="20.375" customWidth="1"/>
+    <col min="5" max="5" width="34.875" customWidth="1"/>
+    <col min="6" max="6" width="23.125" customWidth="1"/>
+    <col min="7" max="7" width="17.25" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="8" spans="3:7">
+      <c r="C8" s="19" t="s">
+        <v>58</v>
+      </c>
+      <c r="D8" s="19" t="s">
+        <v>59</v>
+      </c>
+      <c r="E8" s="19" t="s">
+        <v>60</v>
+      </c>
+      <c r="F8" s="19" t="s">
+        <v>61</v>
+      </c>
+      <c r="G8" s="19" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="9" spans="3:7">
+      <c r="C9" s="20" t="s">
+        <v>63</v>
+      </c>
+      <c r="D9" s="20" t="s">
+        <v>64</v>
+      </c>
+      <c r="E9" s="20" t="s">
+        <v>64</v>
+      </c>
+      <c r="F9" s="20" t="s">
+        <v>65</v>
+      </c>
+      <c r="G9" s="20"/>
+    </row>
+    <row r="10" spans="3:7">
+      <c r="C10" s="20" t="s">
+        <v>66</v>
+      </c>
+      <c r="D10" s="20" t="s">
+        <v>64</v>
+      </c>
+      <c r="E10" s="20" t="s">
+        <v>64</v>
+      </c>
+      <c r="F10" s="20" t="s">
+        <v>49</v>
+      </c>
+      <c r="G10" s="20"/>
+    </row>
+    <row r="11" spans="3:7">
+      <c r="C11" s="20"/>
+      <c r="D11" s="20"/>
+      <c r="E11" s="20"/>
+      <c r="F11" s="20"/>
+      <c r="G11" s="20"/>
+    </row>
+    <row r="12" spans="3:7">
+      <c r="C12" s="20"/>
+      <c r="D12" s="20"/>
+      <c r="E12" s="20"/>
+      <c r="F12" s="20"/>
+      <c r="G12" s="20"/>
+    </row>
+    <row r="13" spans="3:7">
+      <c r="C13" s="20"/>
+      <c r="D13" s="20"/>
+      <c r="E13" s="20"/>
+      <c r="F13" s="20"/>
+      <c r="G13" s="20"/>
+    </row>
+    <row r="14" spans="3:7">
+      <c r="C14" s="20"/>
+      <c r="D14" s="20"/>
+      <c r="E14" s="20"/>
+      <c r="F14" s="20"/>
+      <c r="G14" s="20"/>
+    </row>
+    <row r="15" spans="3:7">
+      <c r="C15" s="20"/>
+      <c r="D15" s="20"/>
+      <c r="E15" s="20"/>
+      <c r="F15" s="20"/>
+      <c r="G15" s="20"/>
+    </row>
+    <row r="16" spans="3:7">
+      <c r="C16" s="20"/>
+      <c r="D16" s="20"/>
+      <c r="E16" s="20"/>
+      <c r="F16" s="20"/>
+      <c r="G16" s="20"/>
+    </row>
+    <row r="17" spans="3:7">
+      <c r="C17" s="20"/>
+      <c r="D17" s="20"/>
+      <c r="E17" s="20"/>
+      <c r="F17" s="20"/>
+      <c r="G17" s="20"/>
+    </row>
+    <row r="18" spans="3:7">
+      <c r="C18" s="20"/>
+      <c r="D18" s="20"/>
+      <c r="E18" s="20"/>
+      <c r="F18" s="20"/>
+      <c r="G18" s="20"/>
+    </row>
+    <row r="19" spans="3:7">
+      <c r="C19" s="20"/>
+      <c r="D19" s="20"/>
+      <c r="E19" s="20"/>
+      <c r="F19" s="20"/>
+      <c r="G19" s="20"/>
+    </row>
+    <row r="20" spans="3:7">
+      <c r="C20" s="20"/>
+      <c r="D20" s="20"/>
+      <c r="E20" s="20"/>
+      <c r="F20" s="20"/>
+      <c r="G20" s="20"/>
+    </row>
+    <row r="21" spans="3:7">
+      <c r="C21" s="20"/>
+      <c r="D21" s="20"/>
+      <c r="E21" s="20"/>
+      <c r="F21" s="20"/>
+      <c r="G21" s="20"/>
+    </row>
+    <row r="22" spans="3:7">
+      <c r="C22" s="20"/>
+      <c r="D22" s="20"/>
+      <c r="E22" s="20"/>
+      <c r="F22" s="20"/>
+      <c r="G22" s="20"/>
+    </row>
+    <row r="23" spans="3:7">
+      <c r="C23" s="20"/>
+      <c r="D23" s="20"/>
+      <c r="E23" s="20"/>
+      <c r="F23" s="20"/>
+      <c r="G23" s="20"/>
+    </row>
+    <row r="24" spans="3:7">
+      <c r="C24" s="20"/>
+      <c r="D24" s="20"/>
+      <c r="E24" s="20"/>
+      <c r="F24" s="20"/>
+      <c r="G24" s="20"/>
+    </row>
+    <row r="25" spans="3:7">
+      <c r="C25" s="20"/>
+      <c r="D25" s="20"/>
+      <c r="E25" s="20"/>
+      <c r="F25" s="20"/>
+      <c r="G25" s="20"/>
+    </row>
+    <row r="26" spans="3:7">
+      <c r="C26" s="20"/>
+      <c r="D26" s="20"/>
+      <c r="E26" s="20"/>
+      <c r="F26" s="20"/>
+      <c r="G26" s="20"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:O34"/>
@@ -2666,7 +2878,7 @@
   <sheetData>
     <row r="1" ht="39" customHeight="1" spans="1:15">
       <c r="A1" s="2" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -2680,34 +2892,34 @@
     </row>
     <row r="2" s="1" customFormat="1" ht="46" customHeight="1" spans="1:15">
       <c r="A2" s="5" t="s">
-        <v>59</v>
+        <v>68</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>60</v>
+        <v>69</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>61</v>
+        <v>70</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>63</v>
+        <v>72</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>64</v>
+        <v>73</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>65</v>
+        <v>74</v>
       </c>
       <c r="H2" s="6" t="s">
-        <v>66</v>
+        <v>75</v>
       </c>
       <c r="I2" s="5" t="s">
-        <v>67</v>
+        <v>76</v>
       </c>
       <c r="J2" s="7" t="s">
-        <v>68</v>
+        <v>77</v>
       </c>
       <c r="K2" s="8"/>
       <c r="L2" s="8"/>
@@ -2723,7 +2935,7 @@
         <v>45</v>
       </c>
       <c r="C3" s="12" t="s">
-        <v>69</v>
+        <v>78</v>
       </c>
       <c r="D3" s="12"/>
       <c r="E3" s="12"/>
@@ -2748,7 +2960,7 @@
         <v>1</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>70</v>
+        <v>79</v>
       </c>
       <c r="F4" s="11" t="s">
         <v>18</v>
@@ -2757,7 +2969,7 @@
         <v>49</v>
       </c>
       <c r="H4" s="15" t="s">
-        <v>71</v>
+        <v>80</v>
       </c>
       <c r="I4" s="11" t="s">
         <v>49</v>
@@ -2781,7 +2993,7 @@
         <v>2</v>
       </c>
       <c r="E5" s="16" t="s">
-        <v>72</v>
+        <v>81</v>
       </c>
       <c r="F5" s="11" t="s">
         <v>20</v>
@@ -2812,17 +3024,17 @@
         <v>2</v>
       </c>
       <c r="E6" s="17" t="s">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>74</v>
+        <v>83</v>
       </c>
       <c r="G6" s="11" t="s">
         <v>49</v>
       </c>
       <c r="H6" s="17"/>
       <c r="I6" s="18" t="s">
-        <v>75</v>
+        <v>84</v>
       </c>
       <c r="J6" s="11" t="s">
         <v>46</v>
@@ -2843,17 +3055,17 @@
         <v>2</v>
       </c>
       <c r="E7" s="17" t="s">
-        <v>76</v>
+        <v>85</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>74</v>
+        <v>83</v>
       </c>
       <c r="G7" s="11" t="s">
         <v>49</v>
       </c>
       <c r="H7" s="17"/>
       <c r="I7" s="18" t="s">
-        <v>75</v>
+        <v>84</v>
       </c>
       <c r="J7" s="11" t="s">
         <v>46</v>
@@ -2874,17 +3086,17 @@
         <v>2</v>
       </c>
       <c r="E8" s="17" t="s">
-        <v>77</v>
+        <v>86</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>74</v>
+        <v>83</v>
       </c>
       <c r="G8" s="11" t="s">
         <v>49</v>
       </c>
       <c r="H8" s="17"/>
       <c r="I8" s="18" t="s">
-        <v>75</v>
+        <v>84</v>
       </c>
       <c r="J8" s="11" t="s">
         <v>46</v>
@@ -2905,17 +3117,17 @@
         <v>2</v>
       </c>
       <c r="E9" s="17" t="s">
-        <v>78</v>
+        <v>87</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>74</v>
+        <v>83</v>
       </c>
       <c r="G9" s="11" t="s">
         <v>49</v>
       </c>
       <c r="H9" s="17"/>
       <c r="I9" s="18" t="s">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="J9" s="11" t="s">
         <v>46</v>
@@ -2936,17 +3148,17 @@
         <v>2</v>
       </c>
       <c r="E10" s="17" t="s">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>74</v>
+        <v>83</v>
       </c>
       <c r="G10" s="11" t="s">
         <v>49</v>
       </c>
       <c r="H10" s="17"/>
       <c r="I10" s="18" t="s">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="J10" s="11" t="s">
         <v>46</v>
@@ -2967,17 +3179,17 @@
         <v>2</v>
       </c>
       <c r="E11" s="17" t="s">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="F11" s="11" t="s">
-        <v>74</v>
+        <v>83</v>
       </c>
       <c r="G11" s="11" t="s">
         <v>49</v>
       </c>
       <c r="H11" s="17"/>
       <c r="I11" s="18" t="s">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="J11" s="11" t="s">
         <v>46</v>
@@ -2997,17 +3209,17 @@
         <v>2</v>
       </c>
       <c r="E12" s="17" t="s">
-        <v>82</v>
+        <v>91</v>
       </c>
       <c r="F12" s="11" t="s">
-        <v>74</v>
+        <v>83</v>
       </c>
       <c r="G12" s="11" t="s">
         <v>49</v>
       </c>
       <c r="H12" s="17"/>
       <c r="I12" s="18" t="s">
-        <v>83</v>
+        <v>92</v>
       </c>
       <c r="J12" s="11" t="s">
         <v>46</v>
@@ -3027,17 +3239,17 @@
         <v>2</v>
       </c>
       <c r="E13" s="17" t="s">
-        <v>84</v>
+        <v>93</v>
       </c>
       <c r="F13" s="11" t="s">
-        <v>74</v>
+        <v>83</v>
       </c>
       <c r="G13" s="11" t="s">
         <v>49</v>
       </c>
       <c r="H13" s="17"/>
       <c r="I13" s="18" t="s">
-        <v>83</v>
+        <v>92</v>
       </c>
       <c r="J13" s="11" t="s">
         <v>46</v>
@@ -3057,17 +3269,17 @@
         <v>2</v>
       </c>
       <c r="E14" s="17" t="s">
-        <v>85</v>
+        <v>94</v>
       </c>
       <c r="F14" s="11" t="s">
-        <v>74</v>
+        <v>83</v>
       </c>
       <c r="G14" s="11" t="s">
         <v>49</v>
       </c>
       <c r="H14" s="17"/>
       <c r="I14" s="18" t="s">
-        <v>83</v>
+        <v>92</v>
       </c>
       <c r="J14" s="11" t="s">
         <v>46</v>
@@ -3087,17 +3299,17 @@
         <v>2</v>
       </c>
       <c r="E15" s="17" t="s">
-        <v>86</v>
+        <v>95</v>
       </c>
       <c r="F15" s="11" t="s">
-        <v>74</v>
+        <v>83</v>
       </c>
       <c r="G15" s="11" t="s">
         <v>49</v>
       </c>
       <c r="H15" s="17"/>
       <c r="I15" s="18" t="s">
-        <v>87</v>
+        <v>96</v>
       </c>
       <c r="J15" s="11" t="s">
         <v>46</v>
@@ -3117,17 +3329,17 @@
         <v>2</v>
       </c>
       <c r="E16" s="17" t="s">
-        <v>88</v>
+        <v>97</v>
       </c>
       <c r="F16" s="11" t="s">
-        <v>74</v>
+        <v>83</v>
       </c>
       <c r="G16" s="11" t="s">
         <v>49</v>
       </c>
       <c r="H16" s="17"/>
       <c r="I16" s="18" t="s">
-        <v>87</v>
+        <v>96</v>
       </c>
       <c r="J16" s="11" t="s">
         <v>46</v>
@@ -3147,17 +3359,17 @@
         <v>2</v>
       </c>
       <c r="E17" s="17" t="s">
-        <v>89</v>
+        <v>98</v>
       </c>
       <c r="F17" s="11" t="s">
-        <v>74</v>
+        <v>83</v>
       </c>
       <c r="G17" s="11" t="s">
         <v>49</v>
       </c>
       <c r="H17" s="17"/>
       <c r="I17" s="18" t="s">
-        <v>87</v>
+        <v>96</v>
       </c>
       <c r="J17" s="11" t="s">
         <v>46</v>
@@ -3177,17 +3389,17 @@
         <v>2</v>
       </c>
       <c r="E18" s="17" t="s">
-        <v>90</v>
+        <v>99</v>
       </c>
       <c r="F18" s="11" t="s">
-        <v>74</v>
+        <v>83</v>
       </c>
       <c r="G18" s="11" t="s">
         <v>49</v>
       </c>
       <c r="H18" s="17"/>
       <c r="I18" s="18" t="s">
-        <v>91</v>
+        <v>100</v>
       </c>
       <c r="J18" s="11" t="s">
         <v>46</v>
@@ -3207,17 +3419,17 @@
         <v>2</v>
       </c>
       <c r="E19" s="17" t="s">
-        <v>92</v>
+        <v>101</v>
       </c>
       <c r="F19" s="11" t="s">
-        <v>74</v>
+        <v>83</v>
       </c>
       <c r="G19" s="11" t="s">
         <v>49</v>
       </c>
       <c r="H19" s="17"/>
       <c r="I19" s="18" t="s">
-        <v>91</v>
+        <v>100</v>
       </c>
       <c r="J19" s="11" t="s">
         <v>46</v>
@@ -3237,17 +3449,17 @@
         <v>2</v>
       </c>
       <c r="E20" s="17" t="s">
-        <v>93</v>
+        <v>102</v>
       </c>
       <c r="F20" s="11" t="s">
-        <v>74</v>
+        <v>83</v>
       </c>
       <c r="G20" s="11" t="s">
         <v>49</v>
       </c>
       <c r="H20" s="17"/>
       <c r="I20" s="18" t="s">
-        <v>91</v>
+        <v>100</v>
       </c>
       <c r="J20" s="11" t="s">
         <v>46</v>
@@ -3267,10 +3479,10 @@
         <v>2</v>
       </c>
       <c r="E21" s="17" t="s">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="F21" s="11" t="s">
-        <v>74</v>
+        <v>83</v>
       </c>
       <c r="G21" s="11" t="s">
         <v>49</v>
@@ -3297,10 +3509,10 @@
         <v>2</v>
       </c>
       <c r="E22" s="17" t="s">
-        <v>95</v>
+        <v>104</v>
       </c>
       <c r="F22" s="11" t="s">
-        <v>74</v>
+        <v>83</v>
       </c>
       <c r="G22" s="11" t="s">
         <v>49</v>
@@ -3327,10 +3539,10 @@
         <v>2</v>
       </c>
       <c r="E23" s="17" t="s">
-        <v>96</v>
+        <v>105</v>
       </c>
       <c r="F23" s="11" t="s">
-        <v>74</v>
+        <v>83</v>
       </c>
       <c r="G23" s="11" t="s">
         <v>49</v>
@@ -3357,17 +3569,17 @@
         <v>2</v>
       </c>
       <c r="E24" s="16" t="s">
-        <v>97</v>
+        <v>106</v>
       </c>
       <c r="F24" s="11" t="s">
-        <v>74</v>
+        <v>83</v>
       </c>
       <c r="G24" s="11" t="s">
         <v>49</v>
       </c>
       <c r="H24" s="17"/>
       <c r="I24" s="18" t="s">
-        <v>75</v>
+        <v>84</v>
       </c>
       <c r="J24" s="11" t="s">
         <v>46</v>
@@ -3385,17 +3597,17 @@
         <v>2</v>
       </c>
       <c r="E25" s="16" t="s">
-        <v>98</v>
+        <v>107</v>
       </c>
       <c r="F25" s="11" t="s">
-        <v>74</v>
+        <v>83</v>
       </c>
       <c r="G25" s="11" t="s">
         <v>49</v>
       </c>
       <c r="H25" s="17"/>
       <c r="I25" s="18" t="s">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="J25" s="11" t="s">
         <v>46</v>
@@ -3413,17 +3625,17 @@
         <v>2</v>
       </c>
       <c r="E26" s="16" t="s">
-        <v>99</v>
+        <v>108</v>
       </c>
       <c r="F26" s="11" t="s">
-        <v>74</v>
+        <v>83</v>
       </c>
       <c r="G26" s="11" t="s">
         <v>49</v>
       </c>
       <c r="H26" s="17"/>
       <c r="I26" s="18" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="J26" s="11" t="s">
         <v>46</v>
@@ -3441,17 +3653,17 @@
         <v>2</v>
       </c>
       <c r="E27" s="16" t="s">
-        <v>101</v>
+        <v>110</v>
       </c>
       <c r="F27" s="11" t="s">
-        <v>74</v>
+        <v>83</v>
       </c>
       <c r="G27" s="11" t="s">
         <v>49</v>
       </c>
       <c r="H27" s="17"/>
       <c r="I27" s="18" t="s">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="J27" s="11" t="s">
         <v>46</v>
@@ -3469,17 +3681,17 @@
         <v>2</v>
       </c>
       <c r="E28" s="16" t="s">
-        <v>102</v>
+        <v>111</v>
       </c>
       <c r="F28" s="11" t="s">
-        <v>74</v>
+        <v>83</v>
       </c>
       <c r="G28" s="11" t="s">
         <v>49</v>
       </c>
       <c r="H28" s="17"/>
       <c r="I28" s="18" t="s">
-        <v>83</v>
+        <v>92</v>
       </c>
       <c r="J28" s="11" t="s">
         <v>46</v>
@@ -3497,17 +3709,17 @@
         <v>2</v>
       </c>
       <c r="E29" s="16" t="s">
-        <v>103</v>
+        <v>112</v>
       </c>
       <c r="F29" s="11" t="s">
-        <v>74</v>
+        <v>83</v>
       </c>
       <c r="G29" s="11" t="s">
         <v>49</v>
       </c>
       <c r="H29" s="17"/>
       <c r="I29" s="18" t="s">
-        <v>87</v>
+        <v>96</v>
       </c>
       <c r="J29" s="11" t="s">
         <v>46</v>
@@ -3525,17 +3737,17 @@
         <v>2</v>
       </c>
       <c r="E30" s="16" t="s">
-        <v>104</v>
+        <v>113</v>
       </c>
       <c r="F30" s="11" t="s">
-        <v>74</v>
+        <v>83</v>
       </c>
       <c r="G30" s="11" t="s">
         <v>49</v>
       </c>
       <c r="H30" s="17"/>
       <c r="I30" s="18" t="s">
-        <v>91</v>
+        <v>100</v>
       </c>
       <c r="J30" s="11" t="s">
         <v>46</v>
@@ -3553,10 +3765,10 @@
         <v>2</v>
       </c>
       <c r="E31" s="17" t="s">
-        <v>105</v>
+        <v>114</v>
       </c>
       <c r="F31" s="11" t="s">
-        <v>74</v>
+        <v>83</v>
       </c>
       <c r="G31" s="11" t="s">
         <v>49</v>
@@ -3581,17 +3793,17 @@
         <v>2</v>
       </c>
       <c r="E32" s="17" t="s">
-        <v>106</v>
+        <v>115</v>
       </c>
       <c r="F32" s="11" t="s">
-        <v>74</v>
+        <v>83</v>
       </c>
       <c r="G32" s="11" t="s">
         <v>49</v>
       </c>
       <c r="H32" s="17"/>
       <c r="I32" s="18" t="s">
-        <v>107</v>
+        <v>116</v>
       </c>
       <c r="J32" s="11" t="s">
         <v>46</v>
@@ -3609,17 +3821,17 @@
         <v>2</v>
       </c>
       <c r="E33" s="16" t="s">
-        <v>108</v>
+        <v>117</v>
       </c>
       <c r="F33" s="11" t="s">
-        <v>74</v>
+        <v>83</v>
       </c>
       <c r="G33" s="11" t="s">
         <v>49</v>
       </c>
       <c r="H33" s="17"/>
       <c r="I33" s="18" t="s">
-        <v>109</v>
+        <v>118</v>
       </c>
       <c r="J33" s="11" t="s">
         <v>46</v>
@@ -3637,17 +3849,17 @@
         <v>2</v>
       </c>
       <c r="E34" s="16" t="s">
-        <v>110</v>
+        <v>119</v>
       </c>
       <c r="F34" s="11" t="s">
-        <v>74</v>
+        <v>83</v>
       </c>
       <c r="G34" s="11" t="s">
         <v>49</v>
       </c>
       <c r="H34" s="17"/>
       <c r="I34" s="18" t="s">
-        <v>109</v>
+        <v>118</v>
       </c>
       <c r="J34" s="11" t="s">
         <v>46</v>

</xml_diff>